<commit_message>
docs(bib): add recent 2022-2026 journal papers, download PDFs, and update reference catalog to fortify methodology
</commit_message>
<xml_diff>
--- a/paper/bibliography/referensi_jurnal_modern.xlsx
+++ b/paper/bibliography/referensi_jurnal_modern.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata Jurnal" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,34 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F497D"/>
-        <bgColor rgb="001F497D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F5F9"/>
-        <bgColor rgb="00F2F5F9"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -60,41 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -460,1454 +413,1846 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
-    <col width="54" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-    <col width="54" customWidth="1" min="7" max="7"/>
-    <col width="54" customWidth="1" min="8" max="8"/>
-    <col width="54" customWidth="1" min="9" max="9"/>
-    <col width="54" customWidth="1" min="10" max="10"/>
-    <col width="54" customWidth="1" min="11" max="11"/>
-    <col width="54" customWidth="1" min="12" max="12"/>
-    <col width="54" customWidth="1" min="13" max="13"/>
-    <col width="54" customWidth="1" min="14" max="14"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Kategori</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Penulis</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Tahun</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Sumber_Jurnal</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DOI_Link</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Masalah</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tujuan</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Metode</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Akurasi_Hasil</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Gap_Relevansi_TA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>A Case Study: Using Passive Acoustic Monitoring Devices In A Growing Urban Landscape To Monitor Avian Diversity</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Tim TIFRH Hyderabad</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>2025</v>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>bioRxiv, 10.1101/2025.07.21.665881</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>https://www.biorxiv.org/content/10.1101/2025.07.21.665881v1.full</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Apakah PAM andal &amp; efisien untuk pemantauan avifauna di lanskap kampus perkotaan biodiverse namun minim data</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Menilai efektivitas PAM di kampus TIFRH (200 acre) dibanding survei tradisional</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>17 perekam, ~3900 jam rekaman (Nov 2024-Mar 2025); diproses BirdNET analyzer default</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Rekaman soundscape kampus TIFRH</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>BirdNET default (tanpa fine-tuning lokasi)</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>135 spesies terdeteksi, 59 salah identifikasi -&gt; hanya 56.3% (76 spesies) benar</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Preseden langsung RQ2 &amp; RQ3: model global perlu kalibrasi threshold pada kampus spesifik</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Nasional</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Implementasi Model Transfer Learning Arsitektur ConvNeXt untuk Klasifikasi Suara Burung di Taman Nasional Way Kambas</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Tim peneliti prosiding</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" t="n">
         <v>2025</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Prosiding SainTek, Universitas Terbuka, Vol. 2 No. 1</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>https://conference.ut.ac.id/index.php/saintek/article/view/5073</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Identifikasi &amp; pemantauan populasi burung TN Way Kambas terkendala SDM, biaya, dan kompleksitas keahlian</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Mengimplementasikan transfer learning ConvNeXt untuk klasifikasi suara burung TN Way Kambas &amp; menemukan konfigurasi optimal</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Pendekatan biofoni, ekstraksi Mel Spectrogram, segmentasi klip 5 detik (librosa), dengan/tanpa augmentasi</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Rekaman suara burung TN Way Kambas</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>ConvNeXt (Base) transfer learning</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>71% (dengan augmentasi data)</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Lokasi &amp; arsitektur sama dengan usulan TA; masih closed-set, belum diuji cross-domain ke soundscape lain</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Nasional</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Klasifikasi Jenis Burung Berdasarkan Suara Kicau Menggunakan Ekstraksi MFCC dan BiLSTM</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Tim Komputa</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>2025</v>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Komputa: Jurnal Ilmiah Komputer dan Informatika, Universitas Komputer Indonesia</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>https://ojs.unikom.ac.id/index.php/komputa/article/view/17694</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Penelitian MFCC sebelumnya belum optimal pada parameter lokal &amp; belum memodelkan pola temporal dua arah</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Mengkombinasikan MFCC teroptimasi dengan BiLSTM untuk klasifikasi burung Indonesia</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>MFCC 40 koefisien; augmentasi data (750 -&gt; 3750 sampel); split 80:20</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>10 spesies burung Indonesia</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>BiLSTM</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>98%</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Akurasi tinggi hanya pada closed-set data bersih; kontras dengan tantangan open-set berderau ITERA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Nasional</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Klasifikasi Suara Katak Menggunakan Model Deep Learning</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Tim prosiding SainTek</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" t="n">
         <v>2025</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Prosiding SainTek, Universitas Terbuka</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>https://conference.ut.ac.id/index.php/saintek/article/download/5065/1909/11831</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Identifikasi spesies katak (bioindikator lingkungan) sulit karena keragaman spesies tinggi</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Mengembangkan klasifikasi suara katak berbasis deep learning</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Ekstraksi fitur MFCC; split 80% latih/10% uji/10% validasi; optimasi Adam</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Rekaman suara katak format WAV</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>DenseNet-121 vs DenseNet-169</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Peningkatan hingga 26.75% dibanding metode acuan sebelumnya</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Contoh bioakustik non-burung (Amphibians) di konteks Indonesia; masih closed-set</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>BirdSet: A Large-Scale Dataset for Audio Classification in Avian Bioacoustics</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Rauch, L.; Schwinger, R.; Wirth, M.; Heinrich, R.; Huseljic, D.; Herde, M.; Lange, J.; Kahl, S.; Sick, B.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" t="n">
         <v>2025</v>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>International Conference on Learning Representations (ICLR 2025)</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>https://openreview.net/forum?id=BirdSet_ICLR2025</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Benchmark bioakustik yang ada sebelumnya terfragmentasi, tidak seragam dalam metrik evaluasi, serta kurang mewakili pergeseran domain focal-to-soundscape yang terstandardisasi</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Menyediakan benchmark skala besar terpadu (BirdSet) mencakup multi-spesies, variasi rekaman soundscape, dan protokol benchmarking reproducible</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Standardisasi task focal-to-soundscape transfer, kalibrasi threshold, dan evaluasi multi-label/open-set</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Kompilasi rekaman focal Xeno-Canto + soundscape teranotasi (POW, HSN, SSW, SNE, PER, dll.)</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>ConvNeXt, EfficientNet-B0, ResNet, BirdNET, Perch</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Performa baseline benchmark terdokumentasi lengkap; model berbasis bioakustik mengungguli model generik pada kondisi soundscape</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Membuktikan bahwa pengujian cross-domain focal-to-soundscape sudah menjadi standar riset modern; memperkuat arah TA untuk paired local robustness benchmark</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Domain-Invariant Representation Learning of Bird Sounds</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Peneliti arXiv:2409.08589</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" t="n">
         <v>2024</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>arXiv:2409.08589</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2409.08589</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Domain shift focal-soundscape mempersulit generalisasi model; SupCon sebelumnya hanya diuji focal-ke-focal</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Mengusulkan pembelajaran representasi invarian domain khusus suara burung</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>ProtoCLR (varian supervised contrastive learning berbasis prototipe kelas)</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Split soundscape BIRB (Sierra Nevada, Hawaii, Kolombia, Kosta Rika, dll.)</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>ProtoCLR vs SupCon</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>ProtoCLR meningkatkan generalisasi few-shot classification lintas dataset BIRB</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Memperkuat argumen kebaruan: cross-domain retrieval tahan derau masih riset aktif</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Nasional</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Klasifikasi Jenis Burung Cucak Berdasarkan Suara Menggunakan MFCC Dan Naive Bayes</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Putra, M. R.; Nurdiyansyah, F.; Rahman, A. Y.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" t="n">
         <v>2024</v>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>JURNAL FASILKOM, 14(2), 463-470</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>https://doi.org/10.37859/jf.v14i2.7558</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Identifikasi manual spesies burung famili Pycnonotidae yang bersuara mirip sulit dilakukan</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Mengembangkan sistem klasifikasi suara burung berbasis MFCC &amp; Naive Bayes untuk 5 spesies Pycnonotidae</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Ekstraksi fitur MFCC + klasifikasi Naive Bayes</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>120 data suara burung dari Xeno-Canto</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Naive Bayes</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>52% (terendah) - 90% (tertinggi), bervariasi antarspesies</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Baseline MFCC pada Xeno-Canto Indonesia; hanya diuji pada data focal bersih, belum pada kondisi lapangan berderau</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>BIRB: A Generalization Benchmark for Information Retrieval in Bioacoustics</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Hamer, J.; Triantafillou, E.; Van Merrienboer, B.; Kahl, S.; Klinck, H.; Denton, T.; Dumoulin, V.</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" t="n">
         <v>2023</v>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>arXiv:2312.07439</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2312.07439</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Belum ada benchmark realistis untuk generalisasi/retrieval pada domain bioakustik (fokus riset generalisasi masih di citra)</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Menyusun benchmark retrieval vokalisasi burung dari data soundscape berbekal exemplar focal recording</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Representation learning + nearest-centroid search; exemplar focal untuk retrieval pada korpus target</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Xeno-Canto (upstream) + berbagai dataset soundscape (evaluasi)</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Baseline representation learning (nearest-centroid)</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Metrik berbasis retrieval (mAP/precision/recall per subset); lihat tabel lengkap paper</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Kerangka metodologis paling dekat dengan skema retrieval TA (RQ1-RQ3); acuan metrik mAP@k/Precision@k/Recall@k</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Global birdsong embeddings enable superior transfer learning for bioacoustic classification</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Ghani, B.; Denton, T.; Kahl, S.; Klinck, H.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" t="n">
         <v>2023</v>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Scientific Reports, 13, 22876</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41598-023-49989-z</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Minimnya representasi embedding bioakustik terpadu yang dapat digeneralisasi ke spesies global dengan data rekaman terbatas (low-resource)</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Menghasilkan representasi embedding bioakustik global berkualitas tinggi berbasis transfer learning untuk klasifikasi bioakustik</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Self-supervised/supervised pretraining pada jutaan rekaman burung global dievaluasi via linear probing dan k-NN similarity</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Xeno-Canto global (&gt;10.000 spesies) + soundscape multi-benua</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Global Birdsong Embeddings (Perch/EfficientNet backbones)</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Mengungguli generic audio embeddings secara masif pada seluruh benchmark bioakustik target</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Rujukan langsung untuk representasi R2 (bioacoustic-specific embedding); novelty TA diposisikan pada retrieval robustness bukan pada pembuatan model embedding baru</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Open-Set Recognition: A Good Closed-Set Classifier is All You Need</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Vaze, S.; Han, K.; Vedaldi, A.; Zisserman, A.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" t="n">
         <v>2022</v>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>ICLR 2022</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2110.06207</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Pembuatan arsitektur OOD khusus terlalu kompleks (menggantikan Scheirer 2012)</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Mendemonstrasikan thresholding / kalibrasi simpel sangat efektif untuk Open-Set</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Maximum Softmax Probability (MSP) &amp; Logit Thresholding</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>ImageNet-OOD</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>VGG / ResNet</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>AUROC SOTA pada benchmark open-set standar</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Dasar metodologi kalibrasi open-set / background noise rejection pada TA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>BirdNET: A deep learning solution for avian diversity monitoring</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Kahl, S.; Wood, C. M.; Eibl, M.; Klinck, H.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" t="n">
         <v>2021</v>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Ecological Informatics, 61, 101236</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.ecoinf.2021.101236</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Volume rekaman PAM terlalu besar untuk diidentifikasi manual; model sulit menggeneralisasi ke berbagai kondisi geografis/akustik</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Mengembangkan sistem klasifikasi suara burung berbasis deep learning yang mudah diterapkan luas termasuk pada rekaman lapangan berderau</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>CNN (backbone mirip EfficientNet) atas spektrogram klip 3 detik; deteksi segmen bersuara berbasis kekuatan sinyal; augmentasi domain</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Jutaan rekaman Xeno-Canto + soundscape (termasuk live-stream Sapsucker Woods)</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>BirdNET (EfficientNet-like), &gt;6000 kelas termasuk non-burung</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Top-1 77.7%, AUC 0.974 (primary prediction); turun signifikan pada domain soundscape</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Dasar empiris domain shift focal-soundscape untuk RQ1 &amp; RQ2; sumber resmi representasi R2</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Overview of BirdCLEF 2021: Bird call identification in soundscape recordings</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Panitia BirdCLEF/LifeCLEF</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" t="n">
         <v>2021</v>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>CEUR Workshop Proceedings, Vol-2936</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>https://ceur-ws.org/Vol-2936/paper-123.pdf</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Domain gap antara sampel latih focal berkualitas tinggi dan sampel uji soundscape berderau</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Melaporkan hasil kompetisi identifikasi panggilan burung pada soundscape edisi 2021</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Kompetisi; kombinasi data focal+soundscape berbagai lokasi geografis</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Xeno-Canto + soundscape multi-lokasi (metadata jenis panggilan, kualitas, migrasi)</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Beragam model peserta kompetisi</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Pola konsisten: akurasi soundscape jauh lebih rendah dibanding focal</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Bukti kuantitatif skala-kompetisi untuk urgensi similarity threshold optimal (RQ2)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>FSD50K: an open dataset of human-labeled sound events</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Fonseca, E.; Favory, X.; Pons, J.; Font, F.; Serra, X.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" t="n">
         <v>2021</v>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>IEEE/ACM Transactions on Audio, Speech, and Language Processing</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2010.00475</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Kurangnya dataset evaluasi audio berskala besar yang realistis dan open-source (menggantikan ESC-50)</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Menyediakan benchmark modern skala masif (51k klip) untuk klasifikasi dan retrieval audio</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Koleksi Freesound, anotasi crowdsourcing, label hierarkis</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>FSD50K</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Baseline CNN (VGG-like)</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>mAP ~ 0.54</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Benchmark pengganti standar untuk pengujian model audio generik (R1)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>AST: Audio Spectrogram Transformer</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Gong, Y.; Chung, Y. A.; Glass, J.</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" t="n">
         <v>2021</v>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Interspeech 2021</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2104.01778</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>CNN bergantung pada bias lokalisasi translasi, kurang mampu menangkap konteks temporal panjang audio</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Menerapkan arsitektur attention murni (Transformer) ke domain audio spectrogram</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Vision Transformer (ViT) diaplikasikan pada patch log-mel spectrogram audio</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>AudioSet, ESC-50, SpeechCommands</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>AST (Audio Spectrogram Transformer)</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>mAP 0.459 (SOTA di AudioSet)</t>
         </is>
       </c>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Dasar arsitektur embedding modern tanpa konvolusi sebagai perbandingan R1/R2 masa kini</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>PANNs: Large-Scale Pretrained Audio Neural Networks for Audio Pattern Recognition</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Kong, Q.; Cao, Y.; Iqbal, T.; Wang, Y.; Wang, W.; Plumbley, M. D.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" t="n">
         <v>2020</v>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>IEEE/ACM Transactions on Audio, Speech, and Language Processing, 28, 2880-2894</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/1912.10211</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Minimnya penelitian pretraining audio berskala besar yang representasinya dapat ditransfer ke berbagai tugas</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Mengusulkan PANNs dan mengevaluasi transferabilitas representasinya ke 6 tugas pengenalan pola audio</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Pretraining pada AudioSet (label lemah) memakai berbagai varian CNN termasuk Wavegram-Logmel-CNN</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>AudioSet (527 kategori peristiwa suara)</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>PANNs / Wavegram-Logmel-CNN (CNN14)</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>mAP 0.439 (vs baseline Google 0.317)</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Sumber resmi representasi R1 (generic audio embedding) vs embedding spesifik burung (BirdNET R2) untuk RQ1</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>A Metric Learning Reality Check</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Musgrave, K.; Belongie, S.; Lim, S. N.</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" t="n">
         <v>2020</v>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>ECCV 2020</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2003.08505</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>Evaluasi sistem metrik retrieval sering bias dan tidak adil (menggantikan Manning 2008)</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Menstandarisasi metrik mAP dan Precision@k untuk membandingkan model berbasis embedding</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Evaluasi ketat ulang dengan hyperparameter tuning yang konsisten</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Beragam Dataset Gambar/Audio</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>ResNet</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Mengoreksi klaim akurasi banyak arsitektur</t>
         </is>
       </c>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>Buku suci modern penentuan evaluasi retrieval (mAP@k, Precision@k) di era Deep Learning</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Nasional</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Identifikasi Jenis Anura dengan Bioakustik pada Kawasan Hutan Lindung Sungai Wain, Kalimantan Timur</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Munda, dkk.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" t="n">
         <v>2020</v>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>ULIN: Jurnal Hutan Tropis, Universitas Mulawarman</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>https://e-journals.unmul.ac.id/index.php/UJHT/article/view/11718</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Inventarisasi anura konvensional (survei visual/penangkapan) invasif dan memakan waktu</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Mengidentifikasi jenis anura di Hutan Lindung Sungai Wain via bioakustik non-invasif</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Perekaman suara panggilan lapangan dibandingkan basis pengetahuan variasi suara anura Indonesia</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Rekaman suara panggilan anura lapangan</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Deskriptif-observasional (bukan ML otomatis)</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>Tidak ada metrik ML (identifikasi berbasis pakar)</t>
         </is>
       </c>
-      <c r="N18" s="3" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Preseden penerimaan bioakustik untuk inventarisasi fauna kawasan konservasi Indonesia (RQ3)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Biotic sound SNR influence analysis on acoustic indices</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Chen, L.; Xu, Z.; Zhao, Z.</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" t="n">
         <v>2023</v>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Frontiers in Remote Sensing, Vol. 3, Article 1079223</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>https://doi.org/10.3389/frsen.2022.1079223</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Kerentanan indeks akustik dan representasi bioakustik terhadap derau abiotik dan penurunan rasio sinyal terhadap derau (SNR) di alam liar</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Menganalisis pengaruh penurunan SNR secara sistematis terhadap integritas representasi suara biologis (biotic sound) dan parameter akustik</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Injeksi derau terkontrol (controlled noise injection) pada sinyal suara biologi lintas rentang level SNR (+20 dB hingga negatif) dan evaluasi kurva degradasi</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Rekaman bioakustik satwa liar dengan injeksi derau abiotik buatan terkontrol</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Analisis kuantitatif indeks akustik dan representasi spektral berbasis kurva degradasi SNR</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>Menunjukkan penurunan drastis korelasi dan kestabilan fitur bioakustik saat SNR &lt; 0 dB; memetakan batas toleransi SNR minimum untuk fitur akustik</t>
         </is>
       </c>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>Rujukan metodologis langsung E2: bagaimana representasi audio terdegradasi ketika SNR turun (Clean, 20dB, 10dB, 0dB, -5dB) dan perumusan kurva retensi relatif</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Few-shot bioacoustic event detection at the DCASE 2023 challenge</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Nolasco, I.; Singh, S.; Benetos, E.; Stowell, D.; et al.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" t="n">
         <v>2023</v>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>arXiv:2306.09223 (DCASE 2023 Challenge Workshop)</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>https://doi.org/10.48550/arXiv.2306.09223</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Keterbatasan data latih berlabel pada vokalisasi satwa (few-shot) serta tingginya variabilitas derau latar belakang dan pergeseran domain perekaman lapangan</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Mengevaluasi arsitektur deteksi dan similarity matching bioakustik few-shot di bawah tantangan variasi lingkungan berderau</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Framework few-shot bioacoustic retrieval, perbandingan matching network, adaptasi prototipe, augmentasi derau, dan kalibrasi threshold penolakan false positive</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Multi-species bioacoustic benchmark (rekaman burung dan mamalia)</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Prototypical Networks, ResNet backbones, metric learning similarity matching</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>Baseline F-score dan evaluasi retrieval terdokumentasi; model berbasis adaptasi fitur dan kalibrasi threshold menghasilkan ketahanan superior terhadap false alarm</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>Rujukan metodologis utama E1 (few-shot clean retrieval), E2 (noise injection benchmark), dan E3 (kalibrasi threshold penolakan kueri negatif / open-set)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Internasional</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Deep audio embeddings for vocalisation clustering</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Best, P.; Paris, S.; Glotin, H.; Marxer, R.</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" t="n">
         <v>2023</v>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>PLoS ONE, 18(4), e0283396</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1371/journal.pone.0283396</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Fitur akustik tradisional (hand-crafted) sulit menggeneralisasi variabilitas akustik dan distorsi lingkungan pada vokalisasi satwa liar</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Membandingkan performa representasi deep audio embeddings (pretrained) versus fitur akustik konvensional dalam merepresentasikan dan mengelompokkan suara satwa</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Ekstraksi fitur hand-crafted (MFCC, temporal acoustic features) vs Deep Pretrained Embeddings, evaluasi jarak kosinus dan metrik retrieval/clustering</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Korpus rekaman bioakustik vokalisasi mamalia dan burung</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>Deep Convolutional Audio Embeddings vs Handcrafted Acoustic Feature Descriptors</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>Deep audio embeddings melipatgandakan kualitas klastering dan separabilitas representasi dibanding fitur akustik konvensional (MFCC)</t>
         </is>
       </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>Justifikasi ilmiah fundamental perbandingan R0 (handcrafted MFCC) vs R1 (PANNs generic deep) dan R2 (BirdNET bioacoustic deep) dalam hipotesis H1 dan H2 TA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Single-station passive acoustic monitoring of bird diversity and vocal activity in Cikaniki, Gunung Halimun-Salak National Park, West Java</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ningrum, I. P.; Mulyani, Y. A.; Mardiastuti, A.</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Journal of Wildlife and Conservation Medicine, Vol. 2 No. 1, pp. 32-39 (IPB University)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.29244/jwcm.2.1.32</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Inventarisasi avifauna di hutan hujan pegunungan Indonesia terkendala kanopi lebat dan vegetasi rapat sehingga survei visual (point count) rentan bias dan undercounting spesies elusif atau kanopi tinggi.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Menilai efektivitas Passive Acoustic Monitoring (PAM) stasiun tunggal untuk mendeteksi kekayaan spesies avifauna serta memetakan karakteristik frekuensi dan rentang durasi kicauan burung di Cikaniki, TN Gunung Halimun-Salak.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Perekaman pasif kontinu 15 hari di stasiun tetap; segmentasi audio dan inspeksi spektrogram; analisis rentang frekuensi (Hz), durasi kicauan (detik), dan indeks aktivitas vokal harian.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Rekaman soundscape kontinu 15 hari stasiun Cikaniki (Taman Nasional Gunung Halimun-Salak, Jawa Barat).</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Inspeksi manual pakar bioakustik berbantuan spektrogram Raven Pro.</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Terdeteksi 40 spesies burung lintas guild; rentang frekuensi 617-8.577 Hz; durasi panggilan berkisar 0,15 hingga 34,29 detik; mendeteksi raptor terbang tinggi (Spilornis cheela) yang luput dari pengamatan visual.</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Justifikasi nasional paling mutakhir untuk PAM avifauna Indonesia: membuktikan jendela 5 detik mampu merangkum mayoritas frase kicauan burung Indonesia, serta mendokumentasikan perlunya toleransi derau lingkungan tropis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SEABAD: A Tropical Bird Activity Detection Dataset for Passive Acoustic Monitoring</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Zabidi, M. M. A.; Idris, M. Y. I.; Idris, N.</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>arXiv:2605.20853</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arXiv.2605.20853</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Model bioakustik yang dilatih pada dataset daerah iklim sedang (temperate) gagal menggeneralisasi pada lingkungan tropis Asia Tenggara akibat tingginya keanekaragaman spesies, masking biophoni serangga, dan derau hujan lebat.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Membangun benchmark dan dataset kurasi berskala besar khusus Bird Activity Detection (BAD) untuk monitoring pasif akustik di kawasan tropis Asia Tenggara.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Segmentasi klip audio 3 detik terstandardisasi; kurasi dual-branch menggabungkan rekaman focal Xeno-Canto Asia Tenggara dan klip soundscape lingkungan negatif; audit akurasi label pakar.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>SEABAD (50.000 klip terkurasi audio 16 kHz mono, mencakup 1.677 spesies burung tropis Asia Tenggara).</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>MobileNetV3-Small, ResNet baseline.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Akurasi klasifikasi deteksi aktivitas 99.57% ± 0.25%, AUC 0.9985 ± 0.0002; audit verifikasi kualitas label 97.8% ± 0.9%.</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Rujukan regional Asia Tenggara untuk Gap 1 &amp; Gap 5: memvalidasi metodologi kurasi data audio Xeno-Canto tropis dan membuktikan perlunya pemisahan sinyal vokal dari derau latar soundscape tropis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MyGardenBird: A Machine-Learning-Ready Bird Sound Dataset for Twelve Common Malaysian Birds</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Zabidi, M. M. A.; Idris, M. Y. I.; Idris, N.</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>arXiv:2606.06975</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arXiv.2606.06975</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Kurangnya dataset bioakustik terkurasi rapi dan berstandar machine learning siap pakai untuk spesies burung umum kawasan biogeografi Sundaland / Semenanjung Melayu.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Mengompilasi dan menstandardisasi dataset suara burung siap latih untuk 12 spesies burung umum regional Indo-Malayan dari repositori Xeno-Canto dengan protokol kurasi reproducible.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Ekstraksi rekaman Xeno-Canto, penyaringan kualitas, penghapusan keheningan (silence trimming), normalisasi audio, dan pengujian klasifikasi baseline supervised &amp; transfer learning.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>MyGardenBird (12 spesies burung umum regional Sundaland: Pycnonotidae, Columbidae, Cisticolidae, dll.).</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>CNN backbones, Transfer Learning Audio Classifiers.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Benchmark klasifikasi multi-spesies mencapai akurasi &gt; 88% pada data bersih, namun mengalami degradasi signifikan saat diuji pada rekaman lapangan berderau.</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Menjawab langsung Gap 1: memperkuat justifikasi pemilihan spesies burung umum kawasan Sundaland (yang berbagi taksonomi identik dengan Pulau Sumatra seperti Merbah cerukcuk dan Tekukur) serta memvalidasi protokol pra-pemrosesan audio berbasis repositori Xeno-Canto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Enabling Multi-Species Bird Classification on Low-Power Bioacoustic Loggers</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ciapponi, S.; Mannini, L.; Scanferla, J.; Anderle, M.; Farella, E.</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>arXiv:2509.20103</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arXiv.2509.20103</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Perangkat bioakustik otonom berdaya rendah (AudioMoth) memiliki keterbatasan memori (RAM ≤ 1 MB) dan daya baterai, sehingga tidak mampu menjalankan model deep learning besar (seperti BirdNET) secara real-time di alam liar.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Mengembangkan arsitektur deep learning ultra-ringan (WrenNet) dengan ekstraktor fitur spektral semi-learnable khusus suara burung yang dapat berjalan langsung pada mikrokontroler AudioMoth.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Ekstraksi fitur spektral adaptif bioakustik, kuantisasi INT8, kompresi bobot, dan deployment langsung pada hardware AudioMoth; komparasi efisiensi energi terhadap Raspberry Pi 3B+ dan BirdNET.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Dataset terkurasi pakar 70 spesies burung.</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>WrenNet (Lightweight Convolutional Neural Network on AudioMoth).</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Akurasi 90.8% pada spesies bersuara distingtif dan 70.1% pada tugas penuh 70 spesies; konsumsi energi hanya 77 mJ per inferensi pada AudioMoth (16x lebih hemat daya dibanding BirdNET di Pi).</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Menjawab langsung Gap 3: memvalidasi secara empiris kapabilitas dan limitasi perangkat keras AudioMoth dalam riset bioakustik modern (2025), serta menjustifikasi mengapa inferensi representasi deep learning tingkat lanjut (PANNs/BirdNET) diproses secara terpisah di workstation/cloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ultra-Compact CNN Architectures for Tropical Bird Audio Detection on Microcontrollers</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Zabidi, M. M. A.; Idris, M. Y. I.; Idris, N.</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>arXiv:2607.19721</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arXiv.2607.19721</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Pemantauan akustik pasif biodiversitas tropis terkendala oleh kapasitas penyimpanan dan baterai karena vokalisasi burung hanya menempati kurang dari 10% durasi soundscape kontinu, sementara 90% sisanya adalah keheningan, derau hujan, atau serangga.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Merancang famili arsitektur detector audio ultra-kompak (DrongoNet) untuk mikrokontroler ARM Cortex-M yang berfungsi memfilter segmen non-vokalisasi langsung pada sensor lapangan.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Desain arsitektur CNN 1D/2D kompak, kuantisasi INT8, evaluasi performa deteksi sinyal di bawah derau lingkungan tropis.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Benchmark audio tropis SEABAD (16 kHz mono).</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>DrongoNet-S, DrongoNet-M, DrongoNet-L (&lt; 50k parameter).</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Mencapai AUC hingga 0.985 dengan latensi inferensi di bawah 150 ms dan jejak memori Flash &lt; 64 KB pada mikrokontroler edge.</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Menjawab langsung Gap 3 &amp; Gap 5: memberikan bukti saintifik bahwa soundscape kontinu lapangan didominasi oleh derau non-target (&gt; 90%), membenarkan penundaan evaluasi soundscape mentah tanpa ground-truth dan memvalidasi pendekatan Paired In-Situ Evaluation berbasis injeksi derau fisik ITERA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Computational bioacoustics with deep learning: a review and roadmap</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Stowell, D.</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PeerJ, 10, e13152</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.7717/peerj.13152</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Pergeseran domain bioakustik ke deep learning menghadapi tantangan unik yang berbeda dari speech/computer vision: langkanya anotasi terverifikasi, label lemah pada rekaman alam, interferensi derau lingkungan liar, dan evaluasi open-set.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Menyajikan tinjauan sistematis komprehensif perkembangan deep learning dalam bioakustik komputasi serta merumuskan roadmap arah riset untuk mengatasi tantangan metodologi yang belum terpecahkan.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Tinjauan sistematis metodologi representasi audio, transfer learning, few-shot recognition, segmentasi temporal, kalibrasi threshold, dan evaluasi cross-domain.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Sintesis beragam korpus bioakustik global (Xeno-Canto, DCASE, Bird Audio Detection, AudioSet).</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>CNN, RNN, Transformers, Metric Learning, Prototypical Networks.</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Analisis komparatif arsitektur SOTA; mengidentifikasi degradasi drastis performa saat model dievaluasi di luar domain latih (domain shift) dan merumuskan protokol evaluasi standar.</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Buku babon komputasi bioakustik deep learning modern. Menjustifikasi Gap 2 &amp; Gap 5: pembagian segmen temporal tetap, pentingnya normalisasi amplitudo/energi, tantangan penolakan derau/open-set (E3), dan alasan saintifik mengapa pengujian robustness bertingkat (E1-E5) sangat krusial.</t>
         </is>
       </c>
     </row>

</xml_diff>